<commit_message>
filtrare + calcul idea
</commit_message>
<xml_diff>
--- a/dateTermistori.xlsx
+++ b/dateTermistori.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29912"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WIP\EVR\EVR_terminal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0AEC31C7-8AD3-4C4E-A8B7-0C05811DCF69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E8F2A5-64C0-484F-967E-32C32220C8AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="7740" windowWidth="14610" windowHeight="7845" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foaie1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Temp Pat</t>
   </si>
@@ -50,14 +50,17 @@
     <t>Medie ADC</t>
   </si>
   <si>
-    <t>Timp</t>
+    <t>MedieAdc_filtrat</t>
+  </si>
+  <si>
+    <t>ADC_ideal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -368,16 +371,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E82"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:F82"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -393,8 +397,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>30</v>
       </c>
@@ -407,8 +414,14 @@
       <c r="D2">
         <v>2708</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="E2">
+        <v>2725.3</v>
+      </c>
+      <c r="F2">
+        <v>1824.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>31</v>
       </c>
@@ -421,8 +434,14 @@
       <c r="D3">
         <v>2670</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="E3">
+        <v>2687.6</v>
+      </c>
+      <c r="F3">
+        <v>1781.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>32</v>
       </c>
@@ -435,8 +454,14 @@
       <c r="D4">
         <v>2640</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="E4">
+        <v>2658.4</v>
+      </c>
+      <c r="F4">
+        <v>1738.7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>33</v>
       </c>
@@ -449,8 +474,14 @@
       <c r="D5">
         <v>2605</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="E5">
+        <v>2621.7</v>
+      </c>
+      <c r="F5">
+        <v>1696.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>34</v>
       </c>
@@ -463,8 +494,14 @@
       <c r="D6">
         <v>2575</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="E6">
+        <v>2593</v>
+      </c>
+      <c r="F6">
+        <v>1655</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>35</v>
       </c>
@@ -477,8 +514,14 @@
       <c r="D7">
         <v>2540</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="E7">
+        <v>2558.5</v>
+      </c>
+      <c r="F7">
+        <v>1614</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>36</v>
       </c>
@@ -491,8 +534,14 @@
       <c r="D8">
         <v>2505</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="E8">
+        <v>2521.3000000000002</v>
+      </c>
+      <c r="F8">
+        <v>1573.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>37</v>
       </c>
@@ -505,8 +554,14 @@
       <c r="D9">
         <v>2475</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="E9">
+        <v>2489.4</v>
+      </c>
+      <c r="F9">
+        <v>1533.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>38</v>
       </c>
@@ -519,8 +574,14 @@
       <c r="D10">
         <v>2440</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="E10">
+        <v>2456.1999999999998</v>
+      </c>
+      <c r="F10">
+        <v>1494.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>39</v>
       </c>
@@ -533,8 +594,14 @@
       <c r="D11">
         <v>2405</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="E11">
+        <v>2422.3000000000002</v>
+      </c>
+      <c r="F11">
+        <v>1456.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>40</v>
       </c>
@@ -547,8 +614,14 @@
       <c r="D12">
         <v>2375</v>
       </c>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="E12">
+        <v>2387.8000000000002</v>
+      </c>
+      <c r="F12">
+        <v>1418.8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>41</v>
       </c>
@@ -561,8 +634,14 @@
       <c r="D13">
         <v>2350</v>
       </c>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="E13">
+        <v>2362.8000000000002</v>
+      </c>
+      <c r="F13">
+        <v>1381.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>42</v>
       </c>
@@ -575,8 +654,14 @@
       <c r="D14">
         <v>2315</v>
       </c>
-    </row>
-    <row r="15" spans="1:5">
+      <c r="E14">
+        <v>2329</v>
+      </c>
+      <c r="F14">
+        <v>1345.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>43</v>
       </c>
@@ -589,8 +674,14 @@
       <c r="D15">
         <v>2280</v>
       </c>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="E15">
+        <v>2284.4</v>
+      </c>
+      <c r="F15">
+        <v>1309.9000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>44</v>
       </c>
@@ -603,8 +694,14 @@
       <c r="D16">
         <v>2235</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="E16">
+        <v>2253.4</v>
+      </c>
+      <c r="F16">
+        <v>1275.0999999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>45</v>
       </c>
@@ -617,8 +714,14 @@
       <c r="D17">
         <v>2205</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="E17">
+        <v>2219.6999999999998</v>
+      </c>
+      <c r="F17">
+        <v>1241</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>46</v>
       </c>
@@ -631,8 +734,14 @@
       <c r="D18">
         <v>2170</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="E18">
+        <v>2185.1999999999998</v>
+      </c>
+      <c r="F18">
+        <v>1207.5999999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>47</v>
       </c>
@@ -645,8 +754,14 @@
       <c r="D19">
         <v>2140</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="E19">
+        <v>2154.3000000000002</v>
+      </c>
+      <c r="F19">
+        <v>1174.9000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>48</v>
       </c>
@@ -659,8 +774,14 @@
       <c r="D20">
         <v>2115</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="E20">
+        <v>2128.1999999999998</v>
+      </c>
+      <c r="F20">
+        <v>1143</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>49</v>
       </c>
@@ -673,8 +794,14 @@
       <c r="D21">
         <v>2085</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="E21">
+        <v>2097.6</v>
+      </c>
+      <c r="F21">
+        <v>1111.8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>50</v>
       </c>
@@ -687,8 +814,14 @@
       <c r="D22">
         <v>2045</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="E22">
+        <v>2058.6</v>
+      </c>
+      <c r="F22">
+        <v>1081.4000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>51</v>
       </c>
@@ -701,8 +834,14 @@
       <c r="D23">
         <v>2015</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="E23">
+        <v>2028.2</v>
+      </c>
+      <c r="F23">
+        <v>1051.5999999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>52</v>
       </c>
@@ -715,8 +854,14 @@
       <c r="D24">
         <v>1985</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="E24">
+        <v>1998.5</v>
+      </c>
+      <c r="F24">
+        <v>1022.6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>53</v>
       </c>
@@ -729,8 +874,14 @@
       <c r="D25">
         <v>1955</v>
       </c>
-    </row>
-    <row r="26" spans="1:4">
+      <c r="E25">
+        <v>1967.6</v>
+      </c>
+      <c r="F25">
+        <v>994.28</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>54</v>
       </c>
@@ -743,8 +894,14 @@
       <c r="D26">
         <v>1930</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
+      <c r="E26">
+        <v>1938.7</v>
+      </c>
+      <c r="F26">
+        <v>966.67</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>55</v>
       </c>
@@ -757,8 +914,14 @@
       <c r="D27">
         <v>1900</v>
       </c>
-    </row>
-    <row r="28" spans="1:4">
+      <c r="E27">
+        <v>1909.9</v>
+      </c>
+      <c r="F27">
+        <v>939.77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>56</v>
       </c>
@@ -771,8 +934,14 @@
       <c r="D28">
         <v>1875</v>
       </c>
-    </row>
-    <row r="29" spans="1:4">
+      <c r="E28">
+        <v>1884.2</v>
+      </c>
+      <c r="F28">
+        <v>913.55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>57</v>
       </c>
@@ -785,8 +954,14 @@
       <c r="D29">
         <v>1845</v>
       </c>
-    </row>
-    <row r="30" spans="1:4">
+      <c r="E29">
+        <v>1854.7</v>
+      </c>
+      <c r="F29">
+        <v>888.01</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>58</v>
       </c>
@@ -799,8 +974,14 @@
       <c r="D30">
         <v>1815</v>
       </c>
-    </row>
-    <row r="31" spans="1:4">
+      <c r="E30">
+        <v>1826.4</v>
+      </c>
+      <c r="F30">
+        <v>863.14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>59</v>
       </c>
@@ -813,8 +994,14 @@
       <c r="D31">
         <v>1790</v>
       </c>
-    </row>
-    <row r="32" spans="1:4">
+      <c r="E31">
+        <v>1798.6</v>
+      </c>
+      <c r="F31">
+        <v>838.93</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>60</v>
       </c>
@@ -827,8 +1014,14 @@
       <c r="D32">
         <v>1760</v>
       </c>
-    </row>
-    <row r="33" spans="1:4">
+      <c r="E32">
+        <v>1771.3</v>
+      </c>
+      <c r="F32">
+        <v>815.37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>61</v>
       </c>
@@ -841,8 +1034,14 @@
       <c r="D33">
         <v>1735</v>
       </c>
-    </row>
-    <row r="34" spans="1:4">
+      <c r="E33">
+        <v>1744.6</v>
+      </c>
+      <c r="F33">
+        <v>792.45</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>62</v>
       </c>
@@ -855,8 +1054,14 @@
       <c r="D34">
         <v>1705</v>
       </c>
-    </row>
-    <row r="35" spans="1:4">
+      <c r="E34">
+        <v>1714.9</v>
+      </c>
+      <c r="F34">
+        <v>770.15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>63</v>
       </c>
@@ -869,8 +1074,14 @@
       <c r="D35">
         <v>1680</v>
       </c>
-    </row>
-    <row r="36" spans="1:4">
+      <c r="E35">
+        <v>1689.1</v>
+      </c>
+      <c r="F35">
+        <v>748.46</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>64</v>
       </c>
@@ -883,8 +1094,14 @@
       <c r="D36">
         <v>1655</v>
       </c>
-    </row>
-    <row r="37" spans="1:4">
+      <c r="E36">
+        <v>1661.8</v>
+      </c>
+      <c r="F36">
+        <v>727.38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>65</v>
       </c>
@@ -897,8 +1114,14 @@
       <c r="D37">
         <v>1630</v>
       </c>
-    </row>
-    <row r="38" spans="1:4">
+      <c r="E37">
+        <v>1637.4</v>
+      </c>
+      <c r="F37">
+        <v>706.89</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>66</v>
       </c>
@@ -911,8 +1134,14 @@
       <c r="D38">
         <v>1607</v>
       </c>
-    </row>
-    <row r="39" spans="1:4">
+      <c r="E38">
+        <v>1611.2</v>
+      </c>
+      <c r="F38">
+        <v>686.97</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>67</v>
       </c>
@@ -925,8 +1154,14 @@
       <c r="D39">
         <v>1580</v>
       </c>
-    </row>
-    <row r="40" spans="1:4">
+      <c r="E39">
+        <v>1587.3</v>
+      </c>
+      <c r="F39">
+        <v>667.62</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>68</v>
       </c>
@@ -939,8 +1174,14 @@
       <c r="D40">
         <v>1558</v>
       </c>
-    </row>
-    <row r="41" spans="1:4">
+      <c r="E40">
+        <v>1566.2</v>
+      </c>
+      <c r="F40">
+        <v>648.80999999999995</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>69</v>
       </c>
@@ -953,8 +1194,14 @@
       <c r="D41">
         <v>1533</v>
       </c>
-    </row>
-    <row r="42" spans="1:4">
+      <c r="E41">
+        <v>1532.8</v>
+      </c>
+      <c r="F41">
+        <v>630.54999999999995</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>70</v>
       </c>
@@ -967,8 +1214,14 @@
       <c r="D42">
         <v>1486</v>
       </c>
-    </row>
-    <row r="43" spans="1:4">
+      <c r="E42">
+        <v>1510.7</v>
+      </c>
+      <c r="F42">
+        <v>612.80999999999995</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>71</v>
       </c>
@@ -981,8 +1234,14 @@
       <c r="D43">
         <v>1463</v>
       </c>
-    </row>
-    <row r="44" spans="1:4">
+      <c r="E43">
+        <v>1459.9</v>
+      </c>
+      <c r="F43">
+        <v>595.58000000000004</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>72</v>
       </c>
@@ -995,8 +1254,14 @@
       <c r="D44">
         <v>1419</v>
       </c>
-    </row>
-    <row r="45" spans="1:4">
+      <c r="E44">
+        <v>1432.8</v>
+      </c>
+      <c r="F44">
+        <v>578.86</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>73</v>
       </c>
@@ -1009,8 +1274,14 @@
       <c r="D45">
         <v>1382</v>
       </c>
-    </row>
-    <row r="46" spans="1:4">
+      <c r="E45">
+        <v>1401.1</v>
+      </c>
+      <c r="F45">
+        <v>562.62</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>74</v>
       </c>
@@ -1023,8 +1294,14 @@
       <c r="D46">
         <v>1304</v>
       </c>
-    </row>
-    <row r="47" spans="1:4">
+      <c r="E46">
+        <v>1386.2</v>
+      </c>
+      <c r="F46">
+        <v>546.85</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>75</v>
       </c>
@@ -1037,8 +1314,14 @@
       <c r="D47">
         <v>1365</v>
       </c>
-    </row>
-    <row r="48" spans="1:4">
+      <c r="E47">
+        <v>1317.8</v>
+      </c>
+      <c r="F47">
+        <v>531.54999999999995</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>76</v>
       </c>
@@ -1051,8 +1334,14 @@
       <c r="D48">
         <v>1270</v>
       </c>
-    </row>
-    <row r="49" spans="1:4">
+      <c r="E48">
+        <v>1279.5999999999999</v>
+      </c>
+      <c r="F48">
+        <v>516.70000000000005</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>77</v>
       </c>
@@ -1065,8 +1354,14 @@
       <c r="D49">
         <v>1255</v>
       </c>
-    </row>
-    <row r="50" spans="1:4">
+      <c r="E49">
+        <v>1255.2</v>
+      </c>
+      <c r="F49">
+        <v>502.29</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>78</v>
       </c>
@@ -1079,8 +1374,14 @@
       <c r="D50">
         <v>1227</v>
       </c>
-    </row>
-    <row r="51" spans="1:4">
+      <c r="E50">
+        <v>1226.5999999999999</v>
+      </c>
+      <c r="F50">
+        <v>488.3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>79</v>
       </c>
@@ -1093,8 +1394,14 @@
       <c r="D51">
         <v>1174</v>
       </c>
-    </row>
-    <row r="52" spans="1:4">
+      <c r="E51">
+        <v>1177.4000000000001</v>
+      </c>
+      <c r="F51">
+        <v>474.73</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>80</v>
       </c>
@@ -1107,8 +1414,14 @@
       <c r="D52">
         <v>1158</v>
       </c>
-    </row>
-    <row r="53" spans="1:4">
+      <c r="E52">
+        <v>1161.2</v>
+      </c>
+      <c r="F52">
+        <v>461.56</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>81</v>
       </c>
@@ -1121,8 +1434,14 @@
       <c r="D53">
         <v>1133</v>
       </c>
-    </row>
-    <row r="54" spans="1:4">
+      <c r="E53">
+        <v>1134.9000000000001</v>
+      </c>
+      <c r="F53">
+        <v>448.79</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>82</v>
       </c>
@@ -1135,8 +1454,14 @@
       <c r="D54">
         <v>1119</v>
       </c>
-    </row>
-    <row r="55" spans="1:4">
+      <c r="E54">
+        <v>1121.7</v>
+      </c>
+      <c r="F54">
+        <v>436.39</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>83</v>
       </c>
@@ -1149,8 +1474,14 @@
       <c r="D55">
         <v>1106</v>
       </c>
-    </row>
-    <row r="56" spans="1:4">
+      <c r="E55">
+        <v>1108.5</v>
+      </c>
+      <c r="F55">
+        <v>424.36</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>84</v>
       </c>
@@ -1163,8 +1494,14 @@
       <c r="D56">
         <v>1095</v>
       </c>
-    </row>
-    <row r="57" spans="1:4">
+      <c r="E56">
+        <v>1097.5999999999999</v>
+      </c>
+      <c r="F56">
+        <v>412.69</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>85</v>
       </c>
@@ -1177,8 +1514,14 @@
       <c r="D57">
         <v>1082</v>
       </c>
-    </row>
-    <row r="58" spans="1:4">
+      <c r="E57">
+        <v>1083.8</v>
+      </c>
+      <c r="F57">
+        <v>401.38</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>86</v>
       </c>
@@ -1191,8 +1534,14 @@
       <c r="D58">
         <v>1072</v>
       </c>
-    </row>
-    <row r="59" spans="1:4">
+      <c r="E58">
+        <v>1074.9000000000001</v>
+      </c>
+      <c r="F58">
+        <v>390.39</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>87</v>
       </c>
@@ -1205,8 +1554,14 @@
       <c r="D59">
         <v>1061</v>
       </c>
-    </row>
-    <row r="60" spans="1:4">
+      <c r="E59">
+        <v>1063.3</v>
+      </c>
+      <c r="F59">
+        <v>379.74</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>88</v>
       </c>
@@ -1219,8 +1574,14 @@
       <c r="D60">
         <v>1050</v>
       </c>
-    </row>
-    <row r="61" spans="1:4">
+      <c r="E60">
+        <v>1052.2</v>
+      </c>
+      <c r="F60">
+        <v>369.41</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>89</v>
       </c>
@@ -1233,8 +1594,14 @@
       <c r="D61">
         <v>1037</v>
       </c>
-    </row>
-    <row r="62" spans="1:4">
+      <c r="E61">
+        <v>1040.2</v>
+      </c>
+      <c r="F61">
+        <v>359.38</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>90</v>
       </c>
@@ -1247,8 +1614,14 @@
       <c r="D62">
         <v>1023</v>
       </c>
-    </row>
-    <row r="63" spans="1:4">
+      <c r="E62">
+        <v>1025.3</v>
+      </c>
+      <c r="F62">
+        <v>349.66</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>91</v>
       </c>
@@ -1261,8 +1634,14 @@
       <c r="D63">
         <v>1014</v>
       </c>
-    </row>
-    <row r="64" spans="1:4">
+      <c r="E63">
+        <v>1016.1</v>
+      </c>
+      <c r="F63">
+        <v>340.22</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>92</v>
       </c>
@@ -1275,8 +1654,14 @@
       <c r="D64">
         <v>1002</v>
       </c>
-    </row>
-    <row r="65" spans="1:4">
+      <c r="E64">
+        <v>1005.8</v>
+      </c>
+      <c r="F64">
+        <v>331.07</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>93</v>
       </c>
@@ -1289,8 +1674,14 @@
       <c r="D65">
         <v>992</v>
       </c>
-    </row>
-    <row r="66" spans="1:4">
+      <c r="E65">
+        <v>995.61</v>
+      </c>
+      <c r="F65">
+        <v>322.19</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>94</v>
       </c>
@@ -1303,8 +1694,14 @@
       <c r="D66">
         <v>981</v>
       </c>
-    </row>
-    <row r="67" spans="1:4">
+      <c r="E66">
+        <v>983.24</v>
+      </c>
+      <c r="F66">
+        <v>313.57</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>95</v>
       </c>
@@ -1317,8 +1714,14 @@
       <c r="D67">
         <v>970</v>
       </c>
-    </row>
-    <row r="68" spans="1:4">
+      <c r="E67">
+        <v>972.46</v>
+      </c>
+      <c r="F67">
+        <v>305.22000000000003</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>96</v>
       </c>
@@ -1331,8 +1734,14 @@
       <c r="D68">
         <v>960</v>
       </c>
-    </row>
-    <row r="69" spans="1:4">
+      <c r="E68">
+        <v>963.86</v>
+      </c>
+      <c r="F68">
+        <v>297.11</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>97</v>
       </c>
@@ -1345,8 +1754,14 @@
       <c r="D69">
         <v>950</v>
       </c>
-    </row>
-    <row r="70" spans="1:4">
+      <c r="E69">
+        <v>953.79</v>
+      </c>
+      <c r="F69">
+        <v>289.24</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>98</v>
       </c>
@@ -1359,8 +1774,14 @@
       <c r="D70">
         <v>941</v>
       </c>
-    </row>
-    <row r="71" spans="1:4">
+      <c r="E70">
+        <v>943.54</v>
+      </c>
+      <c r="F70">
+        <v>281.61</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>99</v>
       </c>
@@ -1373,8 +1794,14 @@
       <c r="D71">
         <v>929</v>
       </c>
-    </row>
-    <row r="72" spans="1:4">
+      <c r="E71">
+        <v>932.31</v>
+      </c>
+      <c r="F71">
+        <v>274.2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>100</v>
       </c>
@@ -1387,8 +1814,14 @@
       <c r="D72">
         <v>920</v>
       </c>
-    </row>
-    <row r="73" spans="1:4">
+      <c r="E72">
+        <v>922.86</v>
+      </c>
+      <c r="F72">
+        <v>267.01</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>101</v>
       </c>
@@ -1401,8 +1834,14 @@
       <c r="D73">
         <v>911</v>
       </c>
-    </row>
-    <row r="74" spans="1:4">
+      <c r="E73">
+        <v>913.54</v>
+      </c>
+      <c r="F73">
+        <v>260.02999999999997</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>102</v>
       </c>
@@ -1415,8 +1854,14 @@
       <c r="D74">
         <v>900</v>
       </c>
-    </row>
-    <row r="75" spans="1:4">
+      <c r="E74">
+        <v>902.67</v>
+      </c>
+      <c r="F74">
+        <v>253.26</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>103</v>
       </c>
@@ -1429,8 +1874,14 @@
       <c r="D75">
         <v>891</v>
       </c>
-    </row>
-    <row r="76" spans="1:4">
+      <c r="E75">
+        <v>894.42</v>
+      </c>
+      <c r="F75">
+        <v>246.7</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>104</v>
       </c>
@@ -1443,8 +1894,14 @@
       <c r="D76">
         <v>883</v>
       </c>
-    </row>
-    <row r="77" spans="1:4">
+      <c r="E76">
+        <v>886.29</v>
+      </c>
+      <c r="F76">
+        <v>240.32</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>105</v>
       </c>
@@ -1457,8 +1914,14 @@
       <c r="D77">
         <v>873</v>
       </c>
-    </row>
-    <row r="78" spans="1:4">
+      <c r="E77">
+        <v>876.4</v>
+      </c>
+      <c r="F77">
+        <v>234.13</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>106</v>
       </c>
@@ -1471,8 +1934,14 @@
       <c r="D78">
         <v>864</v>
       </c>
-    </row>
-    <row r="79" spans="1:4">
+      <c r="E78">
+        <v>867.89</v>
+      </c>
+      <c r="F78">
+        <v>228.12</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>107</v>
       </c>
@@ -1485,8 +1954,14 @@
       <c r="D79">
         <v>856</v>
       </c>
-    </row>
-    <row r="80" spans="1:4">
+      <c r="E79">
+        <v>859.74</v>
+      </c>
+      <c r="F79">
+        <v>222.29</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>108</v>
       </c>
@@ -1499,8 +1974,14 @@
       <c r="D80">
         <v>849</v>
       </c>
-    </row>
-    <row r="81" spans="1:4">
+      <c r="E80">
+        <v>852</v>
+      </c>
+      <c r="F80">
+        <v>216.63</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>109</v>
       </c>
@@ -1513,8 +1994,14 @@
       <c r="D81">
         <v>841</v>
       </c>
-    </row>
-    <row r="82" spans="1:4">
+      <c r="E81">
+        <v>843.72</v>
+      </c>
+      <c r="F81">
+        <v>211.13</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>110</v>
       </c>
@@ -1526,6 +2013,12 @@
       </c>
       <c r="D82">
         <v>833</v>
+      </c>
+      <c r="E82">
+        <v>836.18</v>
+      </c>
+      <c r="F82">
+        <v>205.79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>